<commit_message>
fix(tests): update test harness paths and synchronize methodology workbooks for unified tables and figures reorganization
</commit_message>
<xml_diff>
--- a/tables and figures/methodology/01_Sample_and_Airport_Selection.xlsx
+++ b/tables and figures/methodology/01_Sample_and_Airport_Selection.xlsx
@@ -14,7 +14,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data_sample_profile" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="top25_network_approach" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="power_of_9_airports" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="post_pandemic_justification" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,31 +78,6 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="000000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -139,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -205,17 +179,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -581,11 +544,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -807,71 +770,39 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Table 1.6</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>post_pandemic_justification</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Post-Pandemic Temporal Demarcation Evaluation (Candidate A vs. Candidate B)</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Comparative evaluation of Candidate A (Mature) vs Candidate B (May 1, 2022 Boundary)</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>6 rows x 3 cols</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Temporal Demarcation</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Table 1.7</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>power_of_9_airports</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>The Nine-Airport Experimental Cohort: Generalizability and Twin Disruption Controls</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Spatial transfer pairs, twin disruption shock absorber controls, and statistical balance</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>5 rows x 5 cols</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Experimental Cohort Design</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Note. Master consolidated tabular dataset corresponding to figures in 01_Sample_and_Airport_Selection. Formatted strictly according to APA Style (7th ed.) with horizontal boundary rules, zero auto-filters, and no background shading.</t>
         </is>
@@ -891,8 +822,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -905,7 +834,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
@@ -1120,7 +1049,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -1282,7 +1211,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -1590,7 +1519,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -1774,7 +1703,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -1980,7 +1909,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
@@ -1999,7 +1928,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Table 1.7</t>
+          <t>Table 1.6</t>
         </is>
       </c>
     </row>
@@ -2177,235 +2106,6 @@
       <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Note. Experimental design and testing logic for the nine-airport cohort, establishing intra-cluster zero-shot generalizability pairs and twin disruption resilience controls.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="25" t="inlineStr">
-        <is>
-          <t>⬅ Return to Table of Contents</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>Table 1.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="27" t="inlineStr">
-        <is>
-          <t>Post-Pandemic Temporal Demarcation Specification and Methodological Justification</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>Demarcation Dimension</t>
-        </is>
-      </c>
-      <c r="B5" s="28" t="inlineStr">
-        <is>
-          <t>Methodological Specification</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr">
-        <is>
-          <t>Empirical Verification &amp; Econometric Metric</t>
-        </is>
-      </c>
-      <c r="D5" s="28" t="inlineStr">
-        <is>
-          <t>Operational Significance</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Demarcation Equilibrium Date</t>
-        </is>
-      </c>
-      <c r="B6" s="29" t="inlineStr">
-        <is>
-          <t>May 1, 2022 (Single Established Boundary)</t>
-        </is>
-      </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>Nationwide rescission of federal transit mask mandates (April 18, 2022)</t>
-        </is>
-      </c>
-      <c r="D6" s="29" t="inlineStr">
-        <is>
-          <t>Restored unconstrained passenger travel behaviors and stable flight bank booking patterns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Structural Parameter Stability</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="inlineStr">
-        <is>
-          <t>Chow Structural Break Test across Boundary</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>F = 1.42 (p = 0.18; fails to reject null of coefficient equality)</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>Statistically confirms model parameter invariance and structural stability across the post-demarcation window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Recursive Residual Convergence</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>Cumulative Sum of Recursive Residuals (CUSUM)</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>Residual trajectories strictly bounded within 95% confidence bands</t>
-        </is>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
-        <is>
-          <t>Guarantees variance convergence with zero structural parameter drift throughout the 44-month longitudinal sequence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>Passenger Load Factor Recovery</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>National Commercial Domestic Seat Utilization</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>84.7% Domestic Passenger Load Factor (A14 benchmark)</t>
-        </is>
-      </c>
-      <c r="D9" s="29" t="inlineStr">
-        <is>
-          <t>Matches 2019 pre-pandemic equilibrium, eliminating artificial COVID-19 demand depression and aircraft groundings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>Commercial Coupling Normalization</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>Longitudinal Flight Schedule to TSA Screening Demand</t>
-        </is>
-      </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>r = 0.553, R^2 = 30.61% (Normalized Post-Recovery Coupling)</t>
-        </is>
-      </c>
-      <c r="D10" s="29" t="inlineStr">
-        <is>
-          <t>Rebounds from artificial pandemic distortion (r = 0.607, R^2 = 36.85%) to genuine commercial schedule-demand equilibrium.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="29" t="inlineStr">
-        <is>
-          <t>Total Longitudinal Horizon</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Continuous Multi-Year Analytical Dataset</t>
-        </is>
-      </c>
-      <c r="C11" s="29" t="inlineStr">
-        <is>
-          <t>44 Continuous Calendar Months (May 1, 2022 to December 31, 2025)</t>
-        </is>
-      </c>
-      <c r="D11" s="29" t="inlineStr">
-        <is>
-          <t>Encompasses 1,341 calendar days and 404,324 multi-facility hourly records across the Top 25 national commercial airport benchmark network.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Partitioning &amp; Operational Embargo</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>Temporal Partition Structure (Train / Val / Holdout)</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>20-Month Train / 12-Month Val / 12-Month Out-of-Time 2025 Holdout</t>
-        </is>
-      </c>
-      <c r="D12" s="30" t="inlineStr">
-        <is>
-          <t>Enforces strict 7-day operational purge embargo buffers to prevent delay cascades from leaking across evaluation splits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="31" t="inlineStr">
-        <is>
-          <t>Note. Methodological specification and empirical verification of the post-pandemic temporal demarcation baseline (May 1, 2022 to December 31, 2025).</t>
         </is>
       </c>
     </row>

</xml_diff>